<commit_message>
Add explicit distributed language scheduling
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/排課母版_v6.xlsx
+++ b/backend/tests/fixtures/排課母版_v6.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="說明" sheetId="1" r:id="R484c6d4973cf4ca9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="學校基本資料" sheetId="2" r:id="R90a07e6299fa4c55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="班級" sheetId="3" r:id="R5f38e37d24ca4409"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="教師與配課" sheetId="4" r:id="R669bcd20ed0a4c0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="場地" sheetId="5" r:id="Rfa7700a98ba94c8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="科目節數" sheetId="6" r:id="Rc7e3c8f30ded4c0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="年段時段" sheetId="7" r:id="R0c0299f754cc4f7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="本土語分組" sheetId="8" r:id="Rb4c5792573e342d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="說明" sheetId="1" r:id="Rb95163a218aa4206"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="學校基本資料" sheetId="2" r:id="R4192f7d822c9449b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="班級" sheetId="3" r:id="R2d9f9e86d0404a3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="教師與配課" sheetId="4" r:id="R8ab217c5a6f143ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="場地" sheetId="5" r:id="Rde7fb6b233bb4d89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="科目節數" sheetId="6" r:id="R599e082a45e341b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="年段時段" sheetId="7" r:id="R8e1cec63d4eb46d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="本土語分組" sheetId="8" r:id="Rdc0b547117bb4243"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +20,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="8">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -64,8 +64,24 @@
       <x:color rgb="FF26745F"/>
       <x:name val="Microsoft JhengHei"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF487B99"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF487B99"/>
+      <x:name val="Microsoft JhengHei"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -92,8 +108,28 @@
         <x:fgColor rgb="FFFFFEFD"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC94F7B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC94F7B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="8">
+  <x:borders count="9">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -151,11 +187,25 @@
         <x:color rgb="FFE7D9DE"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE7CFD8"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE7CFD8"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE7CFD8"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE7CFD8"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="40">
+  <x:cellXfs count="53">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -255,6 +305,33 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -4856,6 +4933,8 @@
     <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="19" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="31" customHeight="1">
@@ -4892,6 +4971,12 @@
       <x:c r="K1" s="30" t="str">
         <x:v>上課方式</x:v>
       </x:c>
+      <x:c r="L1" s="50" t="str">
+        <x:v>安排方式</x:v>
+      </x:c>
+      <x:c r="M1" s="50" t="str">
+        <x:v>可抽離科目</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="35" t="n">
@@ -4925,6 +5010,12 @@
       <x:c r="K2" s="35" t="str">
         <x:v>實體</x:v>
       </x:c>
+      <x:c r="L2" s="52" t="str">
+        <x:v>同年級一起上</x:v>
+      </x:c>
+      <x:c r="M2" s="52" t="str">
+        <x:v>國語文、數學</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
       <x:c r="A3" s="35" t="n">
@@ -4958,6 +5049,12 @@
       <x:c r="K3" s="35" t="str">
         <x:v>實體</x:v>
       </x:c>
+      <x:c r="L3" s="52" t="str">
+        <x:v>同年級一起上</x:v>
+      </x:c>
+      <x:c r="M3" s="52" t="str">
+        <x:v>國語文、數學</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="25" customHeight="1">
       <x:c r="A4" s="35" t="n">
@@ -4992,6 +5089,12 @@
       </x:c>
       <x:c r="K4" s="35" t="str">
         <x:v>直播共學</x:v>
+      </x:c>
+      <x:c r="L4" s="52" t="str">
+        <x:v>同年級一起上</x:v>
+      </x:c>
+      <x:c r="M4" s="52" t="str">
+        <x:v>國語文、數學</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="25" customHeight="1">
@@ -5006,6 +5109,8 @@
       <x:c r="I5" s="35"/>
       <x:c r="J5" s="35"/>
       <x:c r="K5" s="35"/>
+      <x:c r="L5" s="52"/>
+      <x:c r="M5" s="52"/>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
       <x:c r="A6" s="35"/>
@@ -5019,6 +5124,8 @@
       <x:c r="I6" s="35"/>
       <x:c r="J6" s="35"/>
       <x:c r="K6" s="35"/>
+      <x:c r="L6" s="52"/>
+      <x:c r="M6" s="52"/>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="35"/>
@@ -5032,6 +5139,8 @@
       <x:c r="I7" s="35"/>
       <x:c r="J7" s="35"/>
       <x:c r="K7" s="35"/>
+      <x:c r="L7" s="52"/>
+      <x:c r="M7" s="52"/>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
       <x:c r="A8" s="35"/>
@@ -5045,6 +5154,8 @@
       <x:c r="I8" s="35"/>
       <x:c r="J8" s="35"/>
       <x:c r="K8" s="35"/>
+      <x:c r="L8" s="52"/>
+      <x:c r="M8" s="52"/>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
       <x:c r="A9" s="35"/>
@@ -5058,6 +5169,8 @@
       <x:c r="I9" s="35"/>
       <x:c r="J9" s="35"/>
       <x:c r="K9" s="35"/>
+      <x:c r="L9" s="52"/>
+      <x:c r="M9" s="52"/>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
       <x:c r="A10" s="35"/>
@@ -5071,6 +5184,8 @@
       <x:c r="I10" s="35"/>
       <x:c r="J10" s="35"/>
       <x:c r="K10" s="35"/>
+      <x:c r="L10" s="52"/>
+      <x:c r="M10" s="52"/>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
       <x:c r="A11" s="35"/>
@@ -5084,6 +5199,8 @@
       <x:c r="I11" s="35"/>
       <x:c r="J11" s="35"/>
       <x:c r="K11" s="35"/>
+      <x:c r="L11" s="52"/>
+      <x:c r="M11" s="52"/>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
       <x:c r="A12" s="35"/>
@@ -5097,6 +5214,8 @@
       <x:c r="I12" s="35"/>
       <x:c r="J12" s="35"/>
       <x:c r="K12" s="35"/>
+      <x:c r="L12" s="52"/>
+      <x:c r="M12" s="52"/>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
       <x:c r="A13" s="35"/>
@@ -5110,6 +5229,8 @@
       <x:c r="I13" s="35"/>
       <x:c r="J13" s="35"/>
       <x:c r="K13" s="35"/>
+      <x:c r="L13" s="52"/>
+      <x:c r="M13" s="52"/>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
       <x:c r="A14" s="35"/>
@@ -5123,6 +5244,8 @@
       <x:c r="I14" s="35"/>
       <x:c r="J14" s="35"/>
       <x:c r="K14" s="35"/>
+      <x:c r="L14" s="52"/>
+      <x:c r="M14" s="52"/>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
       <x:c r="A15" s="35"/>
@@ -5136,6 +5259,8 @@
       <x:c r="I15" s="35"/>
       <x:c r="J15" s="35"/>
       <x:c r="K15" s="35"/>
+      <x:c r="L15" s="52"/>
+      <x:c r="M15" s="52"/>
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
       <x:c r="A16" s="35"/>
@@ -5149,6 +5274,8 @@
       <x:c r="I16" s="35"/>
       <x:c r="J16" s="35"/>
       <x:c r="K16" s="35"/>
+      <x:c r="L16" s="52"/>
+      <x:c r="M16" s="52"/>
     </x:row>
     <x:row r="17" ht="25" customHeight="1">
       <x:c r="A17" s="35"/>
@@ -5162,6 +5289,8 @@
       <x:c r="I17" s="35"/>
       <x:c r="J17" s="35"/>
       <x:c r="K17" s="35"/>
+      <x:c r="L17" s="52"/>
+      <x:c r="M17" s="52"/>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
       <x:c r="A18" s="35"/>
@@ -5175,6 +5304,8 @@
       <x:c r="I18" s="35"/>
       <x:c r="J18" s="35"/>
       <x:c r="K18" s="35"/>
+      <x:c r="L18" s="52"/>
+      <x:c r="M18" s="52"/>
     </x:row>
     <x:row r="19" ht="25" customHeight="1">
       <x:c r="A19" s="35"/>
@@ -5188,6 +5319,8 @@
       <x:c r="I19" s="35"/>
       <x:c r="J19" s="35"/>
       <x:c r="K19" s="35"/>
+      <x:c r="L19" s="52"/>
+      <x:c r="M19" s="52"/>
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
       <x:c r="A20" s="35"/>
@@ -5201,6 +5334,8 @@
       <x:c r="I20" s="35"/>
       <x:c r="J20" s="35"/>
       <x:c r="K20" s="35"/>
+      <x:c r="L20" s="52"/>
+      <x:c r="M20" s="52"/>
     </x:row>
     <x:row r="21" ht="25" customHeight="1">
       <x:c r="A21" s="35"/>
@@ -5214,6 +5349,8 @@
       <x:c r="I21" s="35"/>
       <x:c r="J21" s="35"/>
       <x:c r="K21" s="35"/>
+      <x:c r="L21" s="52"/>
+      <x:c r="M21" s="52"/>
     </x:row>
     <x:row r="22" ht="25" customHeight="1">
       <x:c r="A22" s="35"/>
@@ -5227,6 +5364,8 @@
       <x:c r="I22" s="35"/>
       <x:c r="J22" s="35"/>
       <x:c r="K22" s="35"/>
+      <x:c r="L22" s="52"/>
+      <x:c r="M22" s="52"/>
     </x:row>
     <x:row r="23" ht="25" customHeight="1">
       <x:c r="A23" s="35"/>
@@ -5240,6 +5379,8 @@
       <x:c r="I23" s="35"/>
       <x:c r="J23" s="35"/>
       <x:c r="K23" s="35"/>
+      <x:c r="L23" s="52"/>
+      <x:c r="M23" s="52"/>
     </x:row>
     <x:row r="24" ht="25" customHeight="1">
       <x:c r="A24" s="35"/>
@@ -5253,6 +5394,8 @@
       <x:c r="I24" s="35"/>
       <x:c r="J24" s="35"/>
       <x:c r="K24" s="35"/>
+      <x:c r="L24" s="52"/>
+      <x:c r="M24" s="52"/>
     </x:row>
     <x:row r="25" ht="25" customHeight="1">
       <x:c r="A25" s="35"/>
@@ -5266,6 +5409,8 @@
       <x:c r="I25" s="35"/>
       <x:c r="J25" s="35"/>
       <x:c r="K25" s="35"/>
+      <x:c r="L25" s="52"/>
+      <x:c r="M25" s="52"/>
     </x:row>
     <x:row r="26" ht="25" customHeight="1">
       <x:c r="A26" s="35"/>
@@ -5279,6 +5424,8 @@
       <x:c r="I26" s="35"/>
       <x:c r="J26" s="35"/>
       <x:c r="K26" s="35"/>
+      <x:c r="L26" s="52"/>
+      <x:c r="M26" s="52"/>
     </x:row>
     <x:row r="27" ht="25" customHeight="1">
       <x:c r="A27" s="35"/>
@@ -5292,6 +5439,8 @@
       <x:c r="I27" s="35"/>
       <x:c r="J27" s="35"/>
       <x:c r="K27" s="35"/>
+      <x:c r="L27" s="52"/>
+      <x:c r="M27" s="52"/>
     </x:row>
     <x:row r="28" ht="25" customHeight="1">
       <x:c r="A28" s="35"/>
@@ -5305,6 +5454,8 @@
       <x:c r="I28" s="35"/>
       <x:c r="J28" s="35"/>
       <x:c r="K28" s="35"/>
+      <x:c r="L28" s="52"/>
+      <x:c r="M28" s="52"/>
     </x:row>
     <x:row r="29" ht="25" customHeight="1">
       <x:c r="A29" s="35"/>
@@ -5318,6 +5469,8 @@
       <x:c r="I29" s="35"/>
       <x:c r="J29" s="35"/>
       <x:c r="K29" s="35"/>
+      <x:c r="L29" s="52"/>
+      <x:c r="M29" s="52"/>
     </x:row>
     <x:row r="30" ht="25" customHeight="1">
       <x:c r="A30" s="35"/>
@@ -5331,6 +5484,8 @@
       <x:c r="I30" s="35"/>
       <x:c r="J30" s="35"/>
       <x:c r="K30" s="35"/>
+      <x:c r="L30" s="52"/>
+      <x:c r="M30" s="52"/>
     </x:row>
     <x:row r="31" ht="25" customHeight="1">
       <x:c r="A31" s="35"/>
@@ -5344,6 +5499,8 @@
       <x:c r="I31" s="35"/>
       <x:c r="J31" s="35"/>
       <x:c r="K31" s="35"/>
+      <x:c r="L31" s="52"/>
+      <x:c r="M31" s="52"/>
     </x:row>
     <x:row r="32" ht="25" customHeight="1">
       <x:c r="A32" s="35"/>
@@ -5357,6 +5514,8 @@
       <x:c r="I32" s="35"/>
       <x:c r="J32" s="35"/>
       <x:c r="K32" s="35"/>
+      <x:c r="L32" s="52"/>
+      <x:c r="M32" s="52"/>
     </x:row>
     <x:row r="33" ht="25" customHeight="1">
       <x:c r="A33" s="35"/>
@@ -5370,6 +5529,8 @@
       <x:c r="I33" s="35"/>
       <x:c r="J33" s="35"/>
       <x:c r="K33" s="35"/>
+      <x:c r="L33" s="52"/>
+      <x:c r="M33" s="52"/>
     </x:row>
     <x:row r="34" ht="25" customHeight="1">
       <x:c r="A34" s="35"/>
@@ -5383,6 +5544,8 @@
       <x:c r="I34" s="35"/>
       <x:c r="J34" s="35"/>
       <x:c r="K34" s="35"/>
+      <x:c r="L34" s="52"/>
+      <x:c r="M34" s="52"/>
     </x:row>
     <x:row r="35" ht="25" customHeight="1">
       <x:c r="A35" s="35"/>
@@ -5396,6 +5559,8 @@
       <x:c r="I35" s="35"/>
       <x:c r="J35" s="35"/>
       <x:c r="K35" s="35"/>
+      <x:c r="L35" s="52"/>
+      <x:c r="M35" s="52"/>
     </x:row>
     <x:row r="36" ht="25" customHeight="1">
       <x:c r="A36" s="35"/>
@@ -5409,6 +5574,8 @@
       <x:c r="I36" s="35"/>
       <x:c r="J36" s="35"/>
       <x:c r="K36" s="35"/>
+      <x:c r="L36" s="52"/>
+      <x:c r="M36" s="52"/>
     </x:row>
     <x:row r="37" ht="25" customHeight="1">
       <x:c r="A37" s="35"/>
@@ -5422,6 +5589,8 @@
       <x:c r="I37" s="35"/>
       <x:c r="J37" s="35"/>
       <x:c r="K37" s="35"/>
+      <x:c r="L37" s="52"/>
+      <x:c r="M37" s="52"/>
     </x:row>
     <x:row r="38" ht="25" customHeight="1">
       <x:c r="A38" s="35"/>
@@ -5435,6 +5604,8 @@
       <x:c r="I38" s="35"/>
       <x:c r="J38" s="35"/>
       <x:c r="K38" s="35"/>
+      <x:c r="L38" s="52"/>
+      <x:c r="M38" s="52"/>
     </x:row>
     <x:row r="39" ht="25" customHeight="1">
       <x:c r="A39" s="35"/>
@@ -5448,6 +5619,8 @@
       <x:c r="I39" s="35"/>
       <x:c r="J39" s="35"/>
       <x:c r="K39" s="35"/>
+      <x:c r="L39" s="52"/>
+      <x:c r="M39" s="52"/>
     </x:row>
     <x:row r="40" ht="25" customHeight="1">
       <x:c r="A40" s="35"/>
@@ -5461,6 +5634,8 @@
       <x:c r="I40" s="35"/>
       <x:c r="J40" s="35"/>
       <x:c r="K40" s="35"/>
+      <x:c r="L40" s="52"/>
+      <x:c r="M40" s="52"/>
     </x:row>
     <x:row r="41" ht="25" customHeight="1">
       <x:c r="A41" s="35"/>
@@ -5474,6 +5649,8 @@
       <x:c r="I41" s="35"/>
       <x:c r="J41" s="35"/>
       <x:c r="K41" s="35"/>
+      <x:c r="L41" s="52"/>
+      <x:c r="M41" s="52"/>
     </x:row>
     <x:row r="42" ht="25" customHeight="1">
       <x:c r="A42" s="35"/>
@@ -5487,6 +5664,8 @@
       <x:c r="I42" s="35"/>
       <x:c r="J42" s="35"/>
       <x:c r="K42" s="35"/>
+      <x:c r="L42" s="52"/>
+      <x:c r="M42" s="52"/>
     </x:row>
     <x:row r="43" ht="25" customHeight="1">
       <x:c r="A43" s="35"/>
@@ -5500,6 +5679,8 @@
       <x:c r="I43" s="35"/>
       <x:c r="J43" s="35"/>
       <x:c r="K43" s="35"/>
+      <x:c r="L43" s="52"/>
+      <x:c r="M43" s="52"/>
     </x:row>
     <x:row r="44" ht="25" customHeight="1">
       <x:c r="A44" s="35"/>
@@ -5513,6 +5694,8 @@
       <x:c r="I44" s="35"/>
       <x:c r="J44" s="35"/>
       <x:c r="K44" s="35"/>
+      <x:c r="L44" s="52"/>
+      <x:c r="M44" s="52"/>
     </x:row>
     <x:row r="45" ht="25" customHeight="1">
       <x:c r="A45" s="35"/>
@@ -5526,6 +5709,8 @@
       <x:c r="I45" s="35"/>
       <x:c r="J45" s="35"/>
       <x:c r="K45" s="35"/>
+      <x:c r="L45" s="52"/>
+      <x:c r="M45" s="52"/>
     </x:row>
     <x:row r="46" ht="25" customHeight="1">
       <x:c r="A46" s="35"/>
@@ -5539,6 +5724,8 @@
       <x:c r="I46" s="35"/>
       <x:c r="J46" s="35"/>
       <x:c r="K46" s="35"/>
+      <x:c r="L46" s="52"/>
+      <x:c r="M46" s="52"/>
     </x:row>
     <x:row r="47" ht="25" customHeight="1">
       <x:c r="A47" s="35"/>
@@ -5552,6 +5739,8 @@
       <x:c r="I47" s="35"/>
       <x:c r="J47" s="35"/>
       <x:c r="K47" s="35"/>
+      <x:c r="L47" s="52"/>
+      <x:c r="M47" s="52"/>
     </x:row>
     <x:row r="48" ht="25" customHeight="1">
       <x:c r="A48" s="35"/>
@@ -5565,6 +5754,8 @@
       <x:c r="I48" s="35"/>
       <x:c r="J48" s="35"/>
       <x:c r="K48" s="35"/>
+      <x:c r="L48" s="52"/>
+      <x:c r="M48" s="52"/>
     </x:row>
     <x:row r="49" ht="25" customHeight="1">
       <x:c r="A49" s="35"/>
@@ -5578,6 +5769,8 @@
       <x:c r="I49" s="35"/>
       <x:c r="J49" s="35"/>
       <x:c r="K49" s="35"/>
+      <x:c r="L49" s="52"/>
+      <x:c r="M49" s="52"/>
     </x:row>
     <x:row r="50" ht="25" customHeight="1">
       <x:c r="A50" s="35"/>
@@ -5591,6 +5784,8 @@
       <x:c r="I50" s="35"/>
       <x:c r="J50" s="35"/>
       <x:c r="K50" s="35"/>
+      <x:c r="L50" s="52"/>
+      <x:c r="M50" s="52"/>
     </x:row>
     <x:row r="51" ht="25" customHeight="1">
       <x:c r="A51" s="35"/>
@@ -5604,6 +5799,8 @@
       <x:c r="I51" s="35"/>
       <x:c r="J51" s="35"/>
       <x:c r="K51" s="35"/>
+      <x:c r="L51" s="52"/>
+      <x:c r="M51" s="52"/>
     </x:row>
     <x:row r="52" ht="25" customHeight="1">
       <x:c r="A52" s="35"/>
@@ -5617,6 +5814,8 @@
       <x:c r="I52" s="35"/>
       <x:c r="J52" s="35"/>
       <x:c r="K52" s="35"/>
+      <x:c r="L52" s="52"/>
+      <x:c r="M52" s="52"/>
     </x:row>
     <x:row r="53" ht="25" customHeight="1">
       <x:c r="A53" s="35"/>
@@ -5630,6 +5829,8 @@
       <x:c r="I53" s="35"/>
       <x:c r="J53" s="35"/>
       <x:c r="K53" s="35"/>
+      <x:c r="L53" s="52"/>
+      <x:c r="M53" s="52"/>
     </x:row>
     <x:row r="54" ht="25" customHeight="1">
       <x:c r="A54" s="35"/>
@@ -5643,6 +5844,8 @@
       <x:c r="I54" s="35"/>
       <x:c r="J54" s="35"/>
       <x:c r="K54" s="35"/>
+      <x:c r="L54" s="52"/>
+      <x:c r="M54" s="52"/>
     </x:row>
     <x:row r="55" ht="25" customHeight="1">
       <x:c r="A55" s="35"/>
@@ -5656,6 +5859,8 @@
       <x:c r="I55" s="35"/>
       <x:c r="J55" s="35"/>
       <x:c r="K55" s="35"/>
+      <x:c r="L55" s="52"/>
+      <x:c r="M55" s="52"/>
     </x:row>
     <x:row r="56" ht="25" customHeight="1">
       <x:c r="A56" s="35"/>
@@ -5669,6 +5874,8 @@
       <x:c r="I56" s="35"/>
       <x:c r="J56" s="35"/>
       <x:c r="K56" s="35"/>
+      <x:c r="L56" s="52"/>
+      <x:c r="M56" s="52"/>
     </x:row>
     <x:row r="57" ht="25" customHeight="1">
       <x:c r="A57" s="35"/>
@@ -5682,6 +5889,8 @@
       <x:c r="I57" s="35"/>
       <x:c r="J57" s="35"/>
       <x:c r="K57" s="35"/>
+      <x:c r="L57" s="52"/>
+      <x:c r="M57" s="52"/>
     </x:row>
     <x:row r="58" ht="25" customHeight="1">
       <x:c r="A58" s="35"/>
@@ -5695,6 +5904,8 @@
       <x:c r="I58" s="35"/>
       <x:c r="J58" s="35"/>
       <x:c r="K58" s="35"/>
+      <x:c r="L58" s="52"/>
+      <x:c r="M58" s="52"/>
     </x:row>
     <x:row r="59" ht="25" customHeight="1">
       <x:c r="A59" s="35"/>
@@ -5708,6 +5919,8 @@
       <x:c r="I59" s="35"/>
       <x:c r="J59" s="35"/>
       <x:c r="K59" s="35"/>
+      <x:c r="L59" s="52"/>
+      <x:c r="M59" s="52"/>
     </x:row>
     <x:row r="60" ht="25" customHeight="1">
       <x:c r="A60" s="35"/>
@@ -5721,6 +5934,8 @@
       <x:c r="I60" s="35"/>
       <x:c r="J60" s="35"/>
       <x:c r="K60" s="35"/>
+      <x:c r="L60" s="52"/>
+      <x:c r="M60" s="52"/>
     </x:row>
     <x:row r="61" ht="25" customHeight="1">
       <x:c r="A61" s="35"/>
@@ -5734,6 +5949,8 @@
       <x:c r="I61" s="35"/>
       <x:c r="J61" s="35"/>
       <x:c r="K61" s="35"/>
+      <x:c r="L61" s="52"/>
+      <x:c r="M61" s="52"/>
     </x:row>
     <x:row r="62" ht="25" customHeight="1">
       <x:c r="A62" s="35"/>
@@ -5747,6 +5964,8 @@
       <x:c r="I62" s="35"/>
       <x:c r="J62" s="35"/>
       <x:c r="K62" s="35"/>
+      <x:c r="L62" s="52"/>
+      <x:c r="M62" s="52"/>
     </x:row>
     <x:row r="63" ht="25" customHeight="1">
       <x:c r="A63" s="35"/>
@@ -5760,6 +5979,8 @@
       <x:c r="I63" s="35"/>
       <x:c r="J63" s="35"/>
       <x:c r="K63" s="35"/>
+      <x:c r="L63" s="52"/>
+      <x:c r="M63" s="52"/>
     </x:row>
     <x:row r="64" ht="25" customHeight="1">
       <x:c r="A64" s="35"/>
@@ -5773,6 +5994,8 @@
       <x:c r="I64" s="35"/>
       <x:c r="J64" s="35"/>
       <x:c r="K64" s="35"/>
+      <x:c r="L64" s="52"/>
+      <x:c r="M64" s="52"/>
     </x:row>
     <x:row r="65" ht="25" customHeight="1">
       <x:c r="A65" s="35"/>
@@ -5786,6 +6009,8 @@
       <x:c r="I65" s="35"/>
       <x:c r="J65" s="35"/>
       <x:c r="K65" s="35"/>
+      <x:c r="L65" s="52"/>
+      <x:c r="M65" s="52"/>
     </x:row>
     <x:row r="66" ht="25" customHeight="1">
       <x:c r="A66" s="35"/>
@@ -5799,6 +6024,8 @@
       <x:c r="I66" s="35"/>
       <x:c r="J66" s="35"/>
       <x:c r="K66" s="35"/>
+      <x:c r="L66" s="52"/>
+      <x:c r="M66" s="52"/>
     </x:row>
     <x:row r="67" ht="25" customHeight="1">
       <x:c r="A67" s="35"/>
@@ -5812,6 +6039,8 @@
       <x:c r="I67" s="35"/>
       <x:c r="J67" s="35"/>
       <x:c r="K67" s="35"/>
+      <x:c r="L67" s="52"/>
+      <x:c r="M67" s="52"/>
     </x:row>
     <x:row r="68" ht="25" customHeight="1">
       <x:c r="A68" s="35"/>
@@ -5825,6 +6054,8 @@
       <x:c r="I68" s="35"/>
       <x:c r="J68" s="35"/>
       <x:c r="K68" s="35"/>
+      <x:c r="L68" s="52"/>
+      <x:c r="M68" s="52"/>
     </x:row>
     <x:row r="69" ht="25" customHeight="1">
       <x:c r="A69" s="35"/>
@@ -5838,6 +6069,8 @@
       <x:c r="I69" s="35"/>
       <x:c r="J69" s="35"/>
       <x:c r="K69" s="35"/>
+      <x:c r="L69" s="52"/>
+      <x:c r="M69" s="52"/>
     </x:row>
     <x:row r="70" ht="25" customHeight="1">
       <x:c r="A70" s="35"/>
@@ -5851,6 +6084,8 @@
       <x:c r="I70" s="35"/>
       <x:c r="J70" s="35"/>
       <x:c r="K70" s="35"/>
+      <x:c r="L70" s="52"/>
+      <x:c r="M70" s="52"/>
     </x:row>
     <x:row r="71" ht="25" customHeight="1">
       <x:c r="A71" s="35"/>
@@ -5864,6 +6099,8 @@
       <x:c r="I71" s="35"/>
       <x:c r="J71" s="35"/>
       <x:c r="K71" s="35"/>
+      <x:c r="L71" s="52"/>
+      <x:c r="M71" s="52"/>
     </x:row>
     <x:row r="72" ht="25" customHeight="1">
       <x:c r="A72" s="35"/>
@@ -5877,6 +6114,8 @@
       <x:c r="I72" s="35"/>
       <x:c r="J72" s="35"/>
       <x:c r="K72" s="35"/>
+      <x:c r="L72" s="52"/>
+      <x:c r="M72" s="52"/>
     </x:row>
     <x:row r="73" ht="25" customHeight="1">
       <x:c r="A73" s="35"/>
@@ -5890,6 +6129,8 @@
       <x:c r="I73" s="35"/>
       <x:c r="J73" s="35"/>
       <x:c r="K73" s="35"/>
+      <x:c r="L73" s="52"/>
+      <x:c r="M73" s="52"/>
     </x:row>
     <x:row r="74" ht="25" customHeight="1">
       <x:c r="A74" s="35"/>
@@ -5903,6 +6144,8 @@
       <x:c r="I74" s="35"/>
       <x:c r="J74" s="35"/>
       <x:c r="K74" s="35"/>
+      <x:c r="L74" s="52"/>
+      <x:c r="M74" s="52"/>
     </x:row>
     <x:row r="75" ht="25" customHeight="1">
       <x:c r="A75" s="35"/>
@@ -5916,6 +6159,8 @@
       <x:c r="I75" s="35"/>
       <x:c r="J75" s="35"/>
       <x:c r="K75" s="35"/>
+      <x:c r="L75" s="52"/>
+      <x:c r="M75" s="52"/>
     </x:row>
     <x:row r="76" ht="25" customHeight="1">
       <x:c r="A76" s="35"/>
@@ -5929,6 +6174,8 @@
       <x:c r="I76" s="35"/>
       <x:c r="J76" s="35"/>
       <x:c r="K76" s="35"/>
+      <x:c r="L76" s="52"/>
+      <x:c r="M76" s="52"/>
     </x:row>
     <x:row r="77" ht="25" customHeight="1">
       <x:c r="A77" s="35"/>
@@ -5942,6 +6189,8 @@
       <x:c r="I77" s="35"/>
       <x:c r="J77" s="35"/>
       <x:c r="K77" s="35"/>
+      <x:c r="L77" s="52"/>
+      <x:c r="M77" s="52"/>
     </x:row>
     <x:row r="78" ht="25" customHeight="1">
       <x:c r="A78" s="35"/>
@@ -5955,6 +6204,8 @@
       <x:c r="I78" s="35"/>
       <x:c r="J78" s="35"/>
       <x:c r="K78" s="35"/>
+      <x:c r="L78" s="52"/>
+      <x:c r="M78" s="52"/>
     </x:row>
     <x:row r="79" ht="25" customHeight="1">
       <x:c r="A79" s="35"/>
@@ -5968,6 +6219,8 @@
       <x:c r="I79" s="35"/>
       <x:c r="J79" s="35"/>
       <x:c r="K79" s="35"/>
+      <x:c r="L79" s="52"/>
+      <x:c r="M79" s="52"/>
     </x:row>
     <x:row r="80" ht="25" customHeight="1">
       <x:c r="A80" s="35"/>
@@ -5981,9 +6234,491 @@
       <x:c r="I80" s="35"/>
       <x:c r="J80" s="35"/>
       <x:c r="K80" s="35"/>
+      <x:c r="L80" s="52"/>
+      <x:c r="M80" s="52"/>
+    </x:row>
+    <x:row r="81">
+      <x:c r="L81" s="52"/>
+      <x:c r="M81" s="52"/>
+    </x:row>
+    <x:row r="82">
+      <x:c r="L82" s="52"/>
+      <x:c r="M82" s="52"/>
+    </x:row>
+    <x:row r="83">
+      <x:c r="L83" s="52"/>
+      <x:c r="M83" s="52"/>
+    </x:row>
+    <x:row r="84">
+      <x:c r="L84" s="52"/>
+      <x:c r="M84" s="52"/>
+    </x:row>
+    <x:row r="85">
+      <x:c r="L85" s="52"/>
+      <x:c r="M85" s="52"/>
+    </x:row>
+    <x:row r="86">
+      <x:c r="L86" s="52"/>
+      <x:c r="M86" s="52"/>
+    </x:row>
+    <x:row r="87">
+      <x:c r="L87" s="52"/>
+      <x:c r="M87" s="52"/>
+    </x:row>
+    <x:row r="88">
+      <x:c r="L88" s="52"/>
+      <x:c r="M88" s="52"/>
+    </x:row>
+    <x:row r="89">
+      <x:c r="L89" s="52"/>
+      <x:c r="M89" s="52"/>
+    </x:row>
+    <x:row r="90">
+      <x:c r="L90" s="52"/>
+      <x:c r="M90" s="52"/>
+    </x:row>
+    <x:row r="91">
+      <x:c r="L91" s="52"/>
+      <x:c r="M91" s="52"/>
+    </x:row>
+    <x:row r="92">
+      <x:c r="L92" s="52"/>
+      <x:c r="M92" s="52"/>
+    </x:row>
+    <x:row r="93">
+      <x:c r="L93" s="52"/>
+      <x:c r="M93" s="52"/>
+    </x:row>
+    <x:row r="94">
+      <x:c r="L94" s="52"/>
+      <x:c r="M94" s="52"/>
+    </x:row>
+    <x:row r="95">
+      <x:c r="L95" s="52"/>
+      <x:c r="M95" s="52"/>
+    </x:row>
+    <x:row r="96">
+      <x:c r="L96" s="52"/>
+      <x:c r="M96" s="52"/>
+    </x:row>
+    <x:row r="97">
+      <x:c r="L97" s="52"/>
+      <x:c r="M97" s="52"/>
+    </x:row>
+    <x:row r="98">
+      <x:c r="L98" s="52"/>
+      <x:c r="M98" s="52"/>
+    </x:row>
+    <x:row r="99">
+      <x:c r="L99" s="52"/>
+      <x:c r="M99" s="52"/>
+    </x:row>
+    <x:row r="100">
+      <x:c r="L100" s="52"/>
+      <x:c r="M100" s="52"/>
+    </x:row>
+    <x:row r="101">
+      <x:c r="L101" s="52"/>
+      <x:c r="M101" s="52"/>
+    </x:row>
+    <x:row r="102">
+      <x:c r="L102" s="52"/>
+      <x:c r="M102" s="52"/>
+    </x:row>
+    <x:row r="103">
+      <x:c r="L103" s="52"/>
+      <x:c r="M103" s="52"/>
+    </x:row>
+    <x:row r="104">
+      <x:c r="L104" s="52"/>
+      <x:c r="M104" s="52"/>
+    </x:row>
+    <x:row r="105">
+      <x:c r="L105" s="52"/>
+      <x:c r="M105" s="52"/>
+    </x:row>
+    <x:row r="106">
+      <x:c r="L106" s="52"/>
+      <x:c r="M106" s="52"/>
+    </x:row>
+    <x:row r="107">
+      <x:c r="L107" s="52"/>
+      <x:c r="M107" s="52"/>
+    </x:row>
+    <x:row r="108">
+      <x:c r="L108" s="52"/>
+      <x:c r="M108" s="52"/>
+    </x:row>
+    <x:row r="109">
+      <x:c r="L109" s="52"/>
+      <x:c r="M109" s="52"/>
+    </x:row>
+    <x:row r="110">
+      <x:c r="L110" s="52"/>
+      <x:c r="M110" s="52"/>
+    </x:row>
+    <x:row r="111">
+      <x:c r="L111" s="52"/>
+      <x:c r="M111" s="52"/>
+    </x:row>
+    <x:row r="112">
+      <x:c r="L112" s="52"/>
+      <x:c r="M112" s="52"/>
+    </x:row>
+    <x:row r="113">
+      <x:c r="L113" s="52"/>
+      <x:c r="M113" s="52"/>
+    </x:row>
+    <x:row r="114">
+      <x:c r="L114" s="52"/>
+      <x:c r="M114" s="52"/>
+    </x:row>
+    <x:row r="115">
+      <x:c r="L115" s="52"/>
+      <x:c r="M115" s="52"/>
+    </x:row>
+    <x:row r="116">
+      <x:c r="L116" s="52"/>
+      <x:c r="M116" s="52"/>
+    </x:row>
+    <x:row r="117">
+      <x:c r="L117" s="52"/>
+      <x:c r="M117" s="52"/>
+    </x:row>
+    <x:row r="118">
+      <x:c r="L118" s="52"/>
+      <x:c r="M118" s="52"/>
+    </x:row>
+    <x:row r="119">
+      <x:c r="L119" s="52"/>
+      <x:c r="M119" s="52"/>
+    </x:row>
+    <x:row r="120">
+      <x:c r="L120" s="52"/>
+      <x:c r="M120" s="52"/>
+    </x:row>
+    <x:row r="121">
+      <x:c r="L121" s="52"/>
+      <x:c r="M121" s="52"/>
+    </x:row>
+    <x:row r="122">
+      <x:c r="L122" s="52"/>
+      <x:c r="M122" s="52"/>
+    </x:row>
+    <x:row r="123">
+      <x:c r="L123" s="52"/>
+      <x:c r="M123" s="52"/>
+    </x:row>
+    <x:row r="124">
+      <x:c r="L124" s="52"/>
+      <x:c r="M124" s="52"/>
+    </x:row>
+    <x:row r="125">
+      <x:c r="L125" s="52"/>
+      <x:c r="M125" s="52"/>
+    </x:row>
+    <x:row r="126">
+      <x:c r="L126" s="52"/>
+      <x:c r="M126" s="52"/>
+    </x:row>
+    <x:row r="127">
+      <x:c r="L127" s="52"/>
+      <x:c r="M127" s="52"/>
+    </x:row>
+    <x:row r="128">
+      <x:c r="L128" s="52"/>
+      <x:c r="M128" s="52"/>
+    </x:row>
+    <x:row r="129">
+      <x:c r="L129" s="52"/>
+      <x:c r="M129" s="52"/>
+    </x:row>
+    <x:row r="130">
+      <x:c r="L130" s="52"/>
+      <x:c r="M130" s="52"/>
+    </x:row>
+    <x:row r="131">
+      <x:c r="L131" s="52"/>
+      <x:c r="M131" s="52"/>
+    </x:row>
+    <x:row r="132">
+      <x:c r="L132" s="52"/>
+      <x:c r="M132" s="52"/>
+    </x:row>
+    <x:row r="133">
+      <x:c r="L133" s="52"/>
+      <x:c r="M133" s="52"/>
+    </x:row>
+    <x:row r="134">
+      <x:c r="L134" s="52"/>
+      <x:c r="M134" s="52"/>
+    </x:row>
+    <x:row r="135">
+      <x:c r="L135" s="52"/>
+      <x:c r="M135" s="52"/>
+    </x:row>
+    <x:row r="136">
+      <x:c r="L136" s="52"/>
+      <x:c r="M136" s="52"/>
+    </x:row>
+    <x:row r="137">
+      <x:c r="L137" s="52"/>
+      <x:c r="M137" s="52"/>
+    </x:row>
+    <x:row r="138">
+      <x:c r="L138" s="52"/>
+      <x:c r="M138" s="52"/>
+    </x:row>
+    <x:row r="139">
+      <x:c r="L139" s="52"/>
+      <x:c r="M139" s="52"/>
+    </x:row>
+    <x:row r="140">
+      <x:c r="L140" s="52"/>
+      <x:c r="M140" s="52"/>
+    </x:row>
+    <x:row r="141">
+      <x:c r="L141" s="52"/>
+      <x:c r="M141" s="52"/>
+    </x:row>
+    <x:row r="142">
+      <x:c r="L142" s="52"/>
+      <x:c r="M142" s="52"/>
+    </x:row>
+    <x:row r="143">
+      <x:c r="L143" s="52"/>
+      <x:c r="M143" s="52"/>
+    </x:row>
+    <x:row r="144">
+      <x:c r="L144" s="52"/>
+      <x:c r="M144" s="52"/>
+    </x:row>
+    <x:row r="145">
+      <x:c r="L145" s="52"/>
+      <x:c r="M145" s="52"/>
+    </x:row>
+    <x:row r="146">
+      <x:c r="L146" s="52"/>
+      <x:c r="M146" s="52"/>
+    </x:row>
+    <x:row r="147">
+      <x:c r="L147" s="52"/>
+      <x:c r="M147" s="52"/>
+    </x:row>
+    <x:row r="148">
+      <x:c r="L148" s="52"/>
+      <x:c r="M148" s="52"/>
+    </x:row>
+    <x:row r="149">
+      <x:c r="L149" s="52"/>
+      <x:c r="M149" s="52"/>
+    </x:row>
+    <x:row r="150">
+      <x:c r="L150" s="52"/>
+      <x:c r="M150" s="52"/>
+    </x:row>
+    <x:row r="151">
+      <x:c r="L151" s="52"/>
+      <x:c r="M151" s="52"/>
+    </x:row>
+    <x:row r="152">
+      <x:c r="L152" s="52"/>
+      <x:c r="M152" s="52"/>
+    </x:row>
+    <x:row r="153">
+      <x:c r="L153" s="52"/>
+      <x:c r="M153" s="52"/>
+    </x:row>
+    <x:row r="154">
+      <x:c r="L154" s="52"/>
+      <x:c r="M154" s="52"/>
+    </x:row>
+    <x:row r="155">
+      <x:c r="L155" s="52"/>
+      <x:c r="M155" s="52"/>
+    </x:row>
+    <x:row r="156">
+      <x:c r="L156" s="52"/>
+      <x:c r="M156" s="52"/>
+    </x:row>
+    <x:row r="157">
+      <x:c r="L157" s="52"/>
+      <x:c r="M157" s="52"/>
+    </x:row>
+    <x:row r="158">
+      <x:c r="L158" s="52"/>
+      <x:c r="M158" s="52"/>
+    </x:row>
+    <x:row r="159">
+      <x:c r="L159" s="52"/>
+      <x:c r="M159" s="52"/>
+    </x:row>
+    <x:row r="160">
+      <x:c r="L160" s="52"/>
+      <x:c r="M160" s="52"/>
+    </x:row>
+    <x:row r="161">
+      <x:c r="L161" s="52"/>
+      <x:c r="M161" s="52"/>
+    </x:row>
+    <x:row r="162">
+      <x:c r="L162" s="52"/>
+      <x:c r="M162" s="52"/>
+    </x:row>
+    <x:row r="163">
+      <x:c r="L163" s="52"/>
+      <x:c r="M163" s="52"/>
+    </x:row>
+    <x:row r="164">
+      <x:c r="L164" s="52"/>
+      <x:c r="M164" s="52"/>
+    </x:row>
+    <x:row r="165">
+      <x:c r="L165" s="52"/>
+      <x:c r="M165" s="52"/>
+    </x:row>
+    <x:row r="166">
+      <x:c r="L166" s="52"/>
+      <x:c r="M166" s="52"/>
+    </x:row>
+    <x:row r="167">
+      <x:c r="L167" s="52"/>
+      <x:c r="M167" s="52"/>
+    </x:row>
+    <x:row r="168">
+      <x:c r="L168" s="52"/>
+      <x:c r="M168" s="52"/>
+    </x:row>
+    <x:row r="169">
+      <x:c r="L169" s="52"/>
+      <x:c r="M169" s="52"/>
+    </x:row>
+    <x:row r="170">
+      <x:c r="L170" s="52"/>
+      <x:c r="M170" s="52"/>
+    </x:row>
+    <x:row r="171">
+      <x:c r="L171" s="52"/>
+      <x:c r="M171" s="52"/>
+    </x:row>
+    <x:row r="172">
+      <x:c r="L172" s="52"/>
+      <x:c r="M172" s="52"/>
+    </x:row>
+    <x:row r="173">
+      <x:c r="L173" s="52"/>
+      <x:c r="M173" s="52"/>
+    </x:row>
+    <x:row r="174">
+      <x:c r="L174" s="52"/>
+      <x:c r="M174" s="52"/>
+    </x:row>
+    <x:row r="175">
+      <x:c r="L175" s="52"/>
+      <x:c r="M175" s="52"/>
+    </x:row>
+    <x:row r="176">
+      <x:c r="L176" s="52"/>
+      <x:c r="M176" s="52"/>
+    </x:row>
+    <x:row r="177">
+      <x:c r="L177" s="52"/>
+      <x:c r="M177" s="52"/>
+    </x:row>
+    <x:row r="178">
+      <x:c r="L178" s="52"/>
+      <x:c r="M178" s="52"/>
+    </x:row>
+    <x:row r="179">
+      <x:c r="L179" s="52"/>
+      <x:c r="M179" s="52"/>
+    </x:row>
+    <x:row r="180">
+      <x:c r="L180" s="52"/>
+      <x:c r="M180" s="52"/>
+    </x:row>
+    <x:row r="181">
+      <x:c r="L181" s="52"/>
+      <x:c r="M181" s="52"/>
+    </x:row>
+    <x:row r="182">
+      <x:c r="L182" s="52"/>
+      <x:c r="M182" s="52"/>
+    </x:row>
+    <x:row r="183">
+      <x:c r="L183" s="52"/>
+      <x:c r="M183" s="52"/>
+    </x:row>
+    <x:row r="184">
+      <x:c r="L184" s="52"/>
+      <x:c r="M184" s="52"/>
+    </x:row>
+    <x:row r="185">
+      <x:c r="L185" s="52"/>
+      <x:c r="M185" s="52"/>
+    </x:row>
+    <x:row r="186">
+      <x:c r="L186" s="52"/>
+      <x:c r="M186" s="52"/>
+    </x:row>
+    <x:row r="187">
+      <x:c r="L187" s="52"/>
+      <x:c r="M187" s="52"/>
+    </x:row>
+    <x:row r="188">
+      <x:c r="L188" s="52"/>
+      <x:c r="M188" s="52"/>
+    </x:row>
+    <x:row r="189">
+      <x:c r="L189" s="52"/>
+      <x:c r="M189" s="52"/>
+    </x:row>
+    <x:row r="190">
+      <x:c r="L190" s="52"/>
+      <x:c r="M190" s="52"/>
+    </x:row>
+    <x:row r="191">
+      <x:c r="L191" s="52"/>
+      <x:c r="M191" s="52"/>
+    </x:row>
+    <x:row r="192">
+      <x:c r="L192" s="52"/>
+      <x:c r="M192" s="52"/>
+    </x:row>
+    <x:row r="193">
+      <x:c r="L193" s="52"/>
+      <x:c r="M193" s="52"/>
+    </x:row>
+    <x:row r="194">
+      <x:c r="L194" s="52"/>
+      <x:c r="M194" s="52"/>
+    </x:row>
+    <x:row r="195">
+      <x:c r="L195" s="52"/>
+      <x:c r="M195" s="52"/>
+    </x:row>
+    <x:row r="196">
+      <x:c r="L196" s="52"/>
+      <x:c r="M196" s="52"/>
+    </x:row>
+    <x:row r="197">
+      <x:c r="L197" s="52"/>
+      <x:c r="M197" s="52"/>
+    </x:row>
+    <x:row r="198">
+      <x:c r="L198" s="52"/>
+      <x:c r="M198" s="52"/>
+    </x:row>
+    <x:row r="199">
+      <x:c r="L199" s="52"/>
+      <x:c r="M199" s="52"/>
+    </x:row>
+    <x:row r="200">
+      <x:c r="L200" s="52"/>
+      <x:c r="M200" s="52"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="4">
+  <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="A2:A80">
       <x:formula1>"1,2,3,4,5,6"</x:formula1>
     </x:dataValidation>
@@ -5996,6 +6731,9 @@
     <x:dataValidation type="list" sqref="K2:K80">
       <x:formula1>"實體,直播共學"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="L2:L200">
+      <x:formula1>"同年級一起上,各語別分開上"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>